<commit_message>
Separacion de perfiles y atomatizacion de creacion
</commit_message>
<xml_diff>
--- a/Resultado_Metas_Procesadas.xlsx
+++ b/Resultado_Metas_Procesadas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW21"/>
+  <dimension ref="A1:AW14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -684,27 +684,35 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+        <v>1694138</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YENNY COROMOTO DIAZ PEREZ</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I2" t="n">
-        <v>9175</v>
+        <v>9640</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>504636</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -716,43 +724,43 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="S2" t="n">
+        <v>39</v>
+      </c>
+      <c r="T2" t="n">
+        <v>30</v>
+      </c>
+      <c r="U2" t="n">
+        <v>4</v>
+      </c>
+      <c r="V2" t="n">
+        <v>4</v>
+      </c>
+      <c r="W2" t="n">
+        <v>3</v>
+      </c>
+      <c r="X2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>2.56%</t>
+        </is>
+      </c>
+      <c r="AB2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="n">
-        <v>1</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>2.56%</t>
         </is>
       </c>
       <c r="AD2" t="n">
@@ -762,31 +770,31 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
-        <v>0</v>
+        <v>504636</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>3784.77</v>
       </c>
       <c r="AH2" t="n">
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>504636</v>
       </c>
       <c r="AJ2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AK2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AM2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AN2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AO2" t="n">
         <v>0</v>
@@ -795,25 +803,25 @@
         <v>0</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0</v>
+        <v>-504636</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>-504636</v>
       </c>
       <c r="AS2" t="n">
-        <v>0</v>
+        <v>-504636</v>
       </c>
       <c r="AT2" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU2" t="n">
-        <v>0</v>
+        <v>5046.36</v>
       </c>
       <c r="AV2" t="n">
-        <v>-0.15</v>
+        <v>-0.25</v>
       </c>
       <c r="AW2" t="n">
-        <v>-0</v>
+        <v>-1261.59</v>
       </c>
     </row>
     <row r="3">
@@ -837,35 +845,31 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1694138</v>
+        <v>1099653</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>YENNY COROMOTO DIAZ PEREZ</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+          <t>ANGELA MIREYA MONTENEGRO ROMERO</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>9640</v>
+        <v>9334</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>42028948.63</v>
       </c>
       <c r="K3" t="n">
-        <v>504636</v>
+        <v>7803091</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>18.56599142818006</v>
       </c>
       <c r="M3" t="n">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -877,43 +881,43 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>-3</v>
+        <v>-11</v>
       </c>
       <c r="S3" t="n">
-        <v>39</v>
+        <v>143</v>
       </c>
       <c r="T3" t="n">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="U3" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="V3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="W3" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="X3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Y3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Z3" t="n">
         <v>0</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>13.29%</t>
         </is>
       </c>
       <c r="AD3" t="n">
@@ -923,31 +927,31 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>504636</v>
+        <v>410689</v>
       </c>
       <c r="AG3" t="n">
-        <v>3784.77</v>
+        <v>54621.63699999999</v>
       </c>
       <c r="AH3" t="n">
-        <v>0</v>
+        <v>18.57</v>
       </c>
       <c r="AI3" t="n">
-        <v>504636</v>
+        <v>7803091</v>
       </c>
       <c r="AJ3" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="AK3" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="AL3" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="AM3" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="AN3" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="AO3" t="n">
         <v>0</v>
@@ -956,25 +960,25 @@
         <v>0</v>
       </c>
       <c r="AQ3" t="n">
-        <v>-504636</v>
+        <v>34225857.63</v>
       </c>
       <c r="AR3" t="n">
-        <v>-504636</v>
+        <v>34225857.63</v>
       </c>
       <c r="AS3" t="n">
-        <v>-504636</v>
+        <v>38428752.49300001</v>
       </c>
       <c r="AT3" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU3" t="n">
-        <v>5046.36</v>
+        <v>78030.90999999999</v>
       </c>
       <c r="AV3" t="n">
-        <v>-0.25</v>
+        <v>-0.3</v>
       </c>
       <c r="AW3" t="n">
-        <v>-1261.59</v>
+        <v>-23409.273</v>
       </c>
     </row>
     <row r="4">
@@ -998,31 +1002,35 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1099653</v>
+        <v>1021104</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ANGELA MIREYA MONTENEGRO ROMERO</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>CARMENZA RONCANCIO GACHANCIPA</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I4" t="n">
-        <v>9334</v>
+        <v>7841</v>
       </c>
       <c r="J4" t="n">
-        <v>42028948.63</v>
+        <v>60143077.08</v>
       </c>
       <c r="K4" t="n">
-        <v>7803091</v>
+        <v>12312160</v>
       </c>
       <c r="L4" t="n">
-        <v>18.56599142818006</v>
+        <v>20.47145007832379</v>
       </c>
       <c r="M4" t="n">
-        <v>96</v>
+        <v>150</v>
       </c>
       <c r="N4" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -1034,77 +1042,77 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="S4" t="n">
-        <v>143</v>
+        <v>232</v>
       </c>
       <c r="T4" t="n">
-        <v>87</v>
+        <v>123</v>
       </c>
       <c r="U4" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="V4" t="n">
+        <v>25</v>
+      </c>
+      <c r="W4" t="n">
         <v>10</v>
       </c>
-      <c r="W4" t="n">
-        <v>11</v>
-      </c>
       <c r="X4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>14.22%</t>
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>13.29%</t>
+          <t>13.36%</t>
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>410689</v>
+        <v>373095.7575757576</v>
       </c>
       <c r="AG4" t="n">
-        <v>54621.63699999999</v>
+        <v>86185.12</v>
       </c>
       <c r="AH4" t="n">
-        <v>18.57</v>
+        <v>20.47</v>
       </c>
       <c r="AI4" t="n">
-        <v>7803091</v>
+        <v>12312160</v>
       </c>
       <c r="AJ4" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="AK4" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="AL4" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="AM4" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="AN4" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="AO4" t="n">
         <v>0</v>
@@ -1113,25 +1121,25 @@
         <v>0</v>
       </c>
       <c r="AQ4" t="n">
-        <v>34225857.63</v>
+        <v>47830917.08</v>
       </c>
       <c r="AR4" t="n">
-        <v>34225857.63</v>
+        <v>47830917.08</v>
       </c>
       <c r="AS4" t="n">
-        <v>38428752.49300001</v>
+        <v>53845224.788</v>
       </c>
       <c r="AT4" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU4" t="n">
-        <v>78030.90999999999</v>
+        <v>123121.6</v>
       </c>
       <c r="AV4" t="n">
         <v>-0.3</v>
       </c>
       <c r="AW4" t="n">
-        <v>-23409.273</v>
+        <v>-36936.47999999999</v>
       </c>
     </row>
     <row r="5">
@@ -1155,11 +1163,11 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1021104</v>
+        <v>800685</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CARMENZA RONCANCIO GACHANCIPA</t>
+          <t>JESSICA ROCIO CORTES PERILLA</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1168,22 +1176,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>7841</v>
+        <v>10168</v>
       </c>
       <c r="J5" t="n">
-        <v>60143077.08</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>12312160</v>
+        <v>370613</v>
       </c>
       <c r="L5" t="n">
-        <v>20.47145007832379</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -1195,43 +1203,43 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>-9</v>
+        <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>232</v>
+        <v>11</v>
       </c>
       <c r="T5" t="n">
-        <v>123</v>
+        <v>8</v>
       </c>
       <c r="U5" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="V5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>14.22%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>13.36%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AD5" t="n">
@@ -1241,31 +1249,31 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
-        <v>373095.7575757576</v>
+        <v>370613</v>
       </c>
       <c r="AG5" t="n">
-        <v>86185.12</v>
+        <v>3520.8235</v>
       </c>
       <c r="AH5" t="n">
-        <v>20.47</v>
+        <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>12312160</v>
+        <v>370613</v>
       </c>
       <c r="AJ5" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="AK5" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="AL5" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="AM5" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="AN5" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="AO5" t="n">
         <v>0</v>
@@ -1274,25 +1282,25 @@
         <v>0</v>
       </c>
       <c r="AQ5" t="n">
-        <v>47830917.08</v>
+        <v>-370613</v>
       </c>
       <c r="AR5" t="n">
-        <v>47830917.08</v>
+        <v>-370613</v>
       </c>
       <c r="AS5" t="n">
-        <v>53845224.788</v>
+        <v>-370613</v>
       </c>
       <c r="AT5" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU5" t="n">
-        <v>123121.6</v>
+        <v>3706.13</v>
       </c>
       <c r="AV5" t="n">
-        <v>-0.3</v>
+        <v>-0.05</v>
       </c>
       <c r="AW5" t="n">
-        <v>-36936.47999999999</v>
+        <v>-185.3065</v>
       </c>
     </row>
     <row r="6">
@@ -1316,26 +1324,22 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>800685</v>
+        <v>1407710</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>JESSICA ROCIO CORTES PERILLA</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+          <t>MIGUEL ANGEL MORENO BAUTISTA</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>10168</v>
+        <v>9678</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>370613</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -1344,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -1356,25 +1360,25 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>11</v>
       </c>
       <c r="T6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U6" t="n">
+        <v>3</v>
+      </c>
+      <c r="V6" t="n">
         <v>2</v>
       </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
       <c r="W6" t="n">
         <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y6" t="n">
         <v>0</v>
@@ -1384,49 +1388,49 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>9.09%</t>
+          <t>18.18%</t>
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>18.18%</t>
         </is>
       </c>
       <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
         <v>1</v>
       </c>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>370613</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>3520.8235</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>370613</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>2</v>
-      </c>
       <c r="AK6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AL6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AM6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AN6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -1435,25 +1439,25 @@
         <v>0</v>
       </c>
       <c r="AQ6" t="n">
-        <v>-370613</v>
+        <v>0</v>
       </c>
       <c r="AR6" t="n">
-        <v>-370613</v>
+        <v>0</v>
       </c>
       <c r="AS6" t="n">
-        <v>-370613</v>
+        <v>0</v>
       </c>
       <c r="AT6" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU6" t="n">
-        <v>3706.13</v>
+        <v>0</v>
       </c>
       <c r="AV6" t="n">
-        <v>-0.05</v>
+        <v>-0.15</v>
       </c>
       <c r="AW6" t="n">
-        <v>-185.3065</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="7">
@@ -1477,31 +1481,35 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1407710</v>
+        <v>1077740</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MIGUEL ANGEL MORENO BAUTISTA</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>LUZ MARY LUNA LEON</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I7" t="n">
-        <v>9678</v>
+        <v>9291</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>31598063.23</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>6063738</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>19.19022047605416</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -1513,77 +1521,77 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="S7" t="n">
+        <v>135</v>
+      </c>
+      <c r="T7" t="n">
+        <v>82</v>
+      </c>
+      <c r="U7" t="n">
+        <v>27</v>
+      </c>
+      <c r="V7" t="n">
         <v>11</v>
       </c>
-      <c r="T7" t="n">
-        <v>4</v>
-      </c>
-      <c r="U7" t="n">
-        <v>3</v>
-      </c>
-      <c r="V7" t="n">
-        <v>2</v>
-      </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>11.11%</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>14</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>10.37%</t>
+        </is>
+      </c>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
         <v>1</v>
       </c>
-      <c r="Y7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>18.18%</t>
-        </is>
-      </c>
-      <c r="AB7" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>18.18%</t>
-        </is>
-      </c>
-      <c r="AD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
       <c r="AF7" t="n">
-        <v>0</v>
+        <v>404249.2</v>
       </c>
       <c r="AG7" t="n">
-        <v>0</v>
+        <v>42446.166</v>
       </c>
       <c r="AH7" t="n">
-        <v>0</v>
+        <v>19.19</v>
       </c>
       <c r="AI7" t="n">
-        <v>0</v>
+        <v>6063738</v>
       </c>
       <c r="AJ7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="AK7" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="AL7" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="AM7" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="AN7" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="AO7" t="n">
         <v>0</v>
@@ -1592,25 +1600,25 @@
         <v>0</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0</v>
+        <v>25534325.23</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>25534325.23</v>
       </c>
       <c r="AS7" t="n">
-        <v>0</v>
+        <v>28694131.553</v>
       </c>
       <c r="AT7" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU7" t="n">
-        <v>0</v>
+        <v>60637.37999999999</v>
       </c>
       <c r="AV7" t="n">
-        <v>-0.15</v>
+        <v>-0.3</v>
       </c>
       <c r="AW7" t="n">
-        <v>-0</v>
+        <v>-18191.214</v>
       </c>
     </row>
     <row r="8">
@@ -1634,27 +1642,35 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+        <v>813431</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Luz Dary Chacon Gaitan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I8" t="n">
-        <v>9718</v>
+        <v>8425</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>77487414.67</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>22759714</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>29.37214268527099</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1666,43 +1682,43 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>133</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="X8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Z8" t="n">
         <v>0</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>12.33%</t>
         </is>
       </c>
       <c r="AD8" t="n">
@@ -1712,31 +1728,31 @@
         <v>0</v>
       </c>
       <c r="AF8" t="n">
-        <v>0</v>
+        <v>812846.9285714285</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>159317.998</v>
       </c>
       <c r="AH8" t="n">
-        <v>0</v>
+        <v>29.37</v>
       </c>
       <c r="AI8" t="n">
-        <v>0</v>
+        <v>22759714</v>
       </c>
       <c r="AJ8" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="AK8" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="AL8" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="AM8" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="AN8" t="n">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="AO8" t="n">
         <v>0</v>
@@ -1745,25 +1761,25 @@
         <v>0</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0</v>
+        <v>54727700.67</v>
       </c>
       <c r="AR8" t="n">
-        <v>0</v>
+        <v>54727700.67</v>
       </c>
       <c r="AS8" t="n">
-        <v>0</v>
+        <v>62476442.13700001</v>
       </c>
       <c r="AT8" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU8" t="n">
-        <v>0</v>
+        <v>227597.14</v>
       </c>
       <c r="AV8" t="n">
-        <v>-0.15</v>
+        <v>-0.3</v>
       </c>
       <c r="AW8" t="n">
-        <v>-0</v>
+        <v>-68279.14199999998</v>
       </c>
     </row>
     <row r="9">
@@ -1787,11 +1803,11 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1077740</v>
+        <v>1297183</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>LUZ MARY LUNA LEON</t>
+          <t>DORA INES BELTRAN GAMBA</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1800,22 +1816,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>9291</v>
+        <v>9948</v>
       </c>
       <c r="J9" t="n">
-        <v>31598063.23</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>6063738</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>19.19022047605416</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="N9" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1827,77 +1843,77 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="S9" t="n">
-        <v>135</v>
+        <v>23</v>
       </c>
       <c r="T9" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="U9" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="V9" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W9" t="n">
+        <v>2</v>
+      </c>
+      <c r="X9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL9" t="n">
         <v>5</v>
       </c>
-      <c r="X9" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>11.11%</t>
-        </is>
-      </c>
-      <c r="AB9" t="n">
-        <v>14</v>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>10.37%</t>
-        </is>
-      </c>
-      <c r="AD9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF9" t="n">
-        <v>404249.2</v>
-      </c>
-      <c r="AG9" t="n">
-        <v>42446.166</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>19.19</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>6063738</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>16</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>18</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>20</v>
-      </c>
       <c r="AM9" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="AN9" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="AO9" t="n">
         <v>0</v>
@@ -1906,25 +1922,25 @@
         <v>0</v>
       </c>
       <c r="AQ9" t="n">
-        <v>25534325.23</v>
+        <v>0</v>
       </c>
       <c r="AR9" t="n">
-        <v>25534325.23</v>
+        <v>0</v>
       </c>
       <c r="AS9" t="n">
-        <v>28694131.553</v>
+        <v>0</v>
       </c>
       <c r="AT9" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU9" t="n">
-        <v>60637.37999999999</v>
+        <v>0</v>
       </c>
       <c r="AV9" t="n">
-        <v>-0.3</v>
+        <v>-0.25</v>
       </c>
       <c r="AW9" t="n">
-        <v>-18191.214</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="10">
@@ -1948,35 +1964,31 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>813431</v>
+        <v>1019466</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Luz Dary Chacon Gaitan</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+          <t>LUZ NANCY ROJAS NEIRA</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>8425</v>
+        <v>9717</v>
       </c>
       <c r="J10" t="n">
-        <v>77487414.67</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>22759714</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>29.37214268527099</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1988,43 +2000,43 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>227</v>
+        <v>18</v>
       </c>
       <c r="T10" t="n">
-        <v>133</v>
+        <v>5</v>
       </c>
       <c r="U10" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="V10" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="W10" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Y10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>5.56%</t>
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>12.33%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="AD10" t="n">
@@ -2034,31 +2046,31 @@
         <v>0</v>
       </c>
       <c r="AF10" t="n">
-        <v>812846.9285714285</v>
+        <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>159317.998</v>
+        <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>29.37</v>
+        <v>0</v>
       </c>
       <c r="AI10" t="n">
-        <v>22759714</v>
+        <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="AK10" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="AL10" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="AM10" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="AN10" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
@@ -2067,25 +2079,25 @@
         <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>54727700.67</v>
+        <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>54727700.67</v>
+        <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>62476442.13700001</v>
+        <v>0</v>
       </c>
       <c r="AT10" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU10" t="n">
-        <v>227597.14</v>
+        <v>0</v>
       </c>
       <c r="AV10" t="n">
-        <v>-0.3</v>
+        <v>-0.15</v>
       </c>
       <c r="AW10" t="n">
-        <v>-68279.14199999998</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="11">
@@ -2109,35 +2121,31 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1297183</v>
+        <v>768496</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>DORA INES BELTRAN GAMBA</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
+          <t>LUZ ADRIANA PAEZ VIGOYA</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>9948</v>
+        <v>8481</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>63767465.56</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>10739821</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>16.84216379886496</v>
       </c>
       <c r="M11" t="n">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -2149,43 +2157,43 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>-2</v>
+        <v>-12</v>
       </c>
       <c r="S11" t="n">
-        <v>23</v>
+        <v>208</v>
       </c>
       <c r="T11" t="n">
-        <v>20</v>
+        <v>133</v>
       </c>
       <c r="U11" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="V11" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="W11" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="X11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="Z11" t="n">
         <v>0</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>10.10%</t>
         </is>
       </c>
       <c r="AD11" t="n">
@@ -2195,31 +2203,31 @@
         <v>0</v>
       </c>
       <c r="AF11" t="n">
-        <v>0</v>
+        <v>511420.0476190476</v>
       </c>
       <c r="AG11" t="n">
-        <v>0</v>
+        <v>75178.74699999999</v>
       </c>
       <c r="AH11" t="n">
-        <v>0</v>
+        <v>16.84</v>
       </c>
       <c r="AI11" t="n">
-        <v>0</v>
+        <v>10739821</v>
       </c>
       <c r="AJ11" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="AK11" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="AL11" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="AM11" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="AN11" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -2228,25 +2236,25 @@
         <v>0</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0</v>
+        <v>53027644.56</v>
       </c>
       <c r="AR11" t="n">
-        <v>0</v>
+        <v>53027644.56</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>59404391.11600001</v>
       </c>
       <c r="AT11" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU11" t="n">
-        <v>0</v>
+        <v>107398.21</v>
       </c>
       <c r="AV11" t="n">
-        <v>-0.25</v>
+        <v>-0.3</v>
       </c>
       <c r="AW11" t="n">
-        <v>-0</v>
+        <v>-32219.46299999999</v>
       </c>
     </row>
     <row r="12">
@@ -2270,12 +2278,20 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+        <v>1741255</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>EVELYN GOMEZ LOZANO</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I12" t="n">
-        <v>8048</v>
+        <v>10223</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -2305,10 +2321,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -2320,7 +2336,7 @@
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y12" t="n">
         <v>0</v>
@@ -2423,12 +2439,20 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+        <v>1665372</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>DORIS ANGARITA</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I13" t="n">
-        <v>10261</v>
+        <v>10260</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -2458,10 +2482,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -2576,27 +2600,35 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+        <v>985990</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>MARIA CRISTINA RUBIO</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ORO</t>
+        </is>
+      </c>
       <c r="I14" t="n">
-        <v>9581</v>
+        <v>9400</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>23747542.18</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1573859</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>6.627460593903027</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -2608,43 +2640,43 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>-2</v>
+        <v>-11</v>
       </c>
       <c r="S14" t="n">
-        <v>7</v>
+        <v>94</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="V14" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="W14" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="X14" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="Y14" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>5.32%</t>
         </is>
       </c>
       <c r="AB14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>5.32%</t>
         </is>
       </c>
       <c r="AD14" t="n">
@@ -2654,31 +2686,31 @@
         <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>0</v>
+        <v>314771.8</v>
       </c>
       <c r="AG14" t="n">
-        <v>0</v>
+        <v>11017.013</v>
       </c>
       <c r="AH14" t="n">
-        <v>0</v>
+        <v>6.63</v>
       </c>
       <c r="AI14" t="n">
-        <v>0</v>
+        <v>1573859</v>
       </c>
       <c r="AJ14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AK14" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AL14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AM14" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="AN14" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="AO14" t="n">
         <v>0</v>
@@ -2687,1127 +2719,24 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0</v>
+        <v>22173683.18</v>
       </c>
       <c r="AR14" t="n">
-        <v>0</v>
+        <v>22173683.18</v>
       </c>
       <c r="AS14" t="n">
-        <v>0</v>
+        <v>24548437.398</v>
       </c>
       <c r="AT14" t="n">
         <v>0.009999999999999998</v>
       </c>
       <c r="AU14" t="n">
-        <v>0</v>
+        <v>15738.59</v>
       </c>
       <c r="AV14" t="n">
-        <v>-0.25</v>
+        <v>-0.3</v>
       </c>
       <c r="AW14" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B15" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>9376</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK15" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>9</v>
-      </c>
-      <c r="AO15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT15" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV15" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AW15" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B16" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>1019466</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>LUZ NANCY ROJAS NEIRA</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>9717</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" t="n">
-        <v>18</v>
-      </c>
-      <c r="T16" t="n">
-        <v>5</v>
-      </c>
-      <c r="U16" t="n">
-        <v>9</v>
-      </c>
-      <c r="V16" t="n">
-        <v>3</v>
-      </c>
-      <c r="W16" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>5.56%</t>
-        </is>
-      </c>
-      <c r="AB16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL16" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM16" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN16" t="n">
-        <v>9</v>
-      </c>
-      <c r="AO16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT16" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AW16" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B17" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>768496</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>LUZ ADRIANA PAEZ VIGOYA</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>8481</v>
-      </c>
-      <c r="J17" t="n">
-        <v>63767465.56</v>
-      </c>
-      <c r="K17" t="n">
-        <v>10739821</v>
-      </c>
-      <c r="L17" t="n">
-        <v>16.84216379886496</v>
-      </c>
-      <c r="M17" t="n">
-        <v>136</v>
-      </c>
-      <c r="N17" t="n">
-        <v>21</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>-12</v>
-      </c>
-      <c r="S17" t="n">
-        <v>208</v>
-      </c>
-      <c r="T17" t="n">
-        <v>133</v>
-      </c>
-      <c r="U17" t="n">
-        <v>40</v>
-      </c>
-      <c r="V17" t="n">
-        <v>14</v>
-      </c>
-      <c r="W17" t="n">
-        <v>12</v>
-      </c>
-      <c r="X17" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>12</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>10.10%</t>
-        </is>
-      </c>
-      <c r="AB17" t="n">
-        <v>21</v>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>10.10%</t>
-        </is>
-      </c>
-      <c r="AD17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>511420.0476190476</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>75178.74699999999</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>10739821</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>22</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>24</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>26</v>
-      </c>
-      <c r="AM17" t="n">
-        <v>28</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>30</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>53027644.56</v>
-      </c>
-      <c r="AR17" t="n">
-        <v>53027644.56</v>
-      </c>
-      <c r="AS17" t="n">
-        <v>59404391.11600001</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU17" t="n">
-        <v>107398.21</v>
-      </c>
-      <c r="AV17" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="AW17" t="n">
-        <v>-32219.46299999999</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B18" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>10255</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="n">
-        <v>1</v>
-      </c>
-      <c r="T18" t="n">
-        <v>1</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" t="n">
-        <v>0</v>
-      </c>
-      <c r="W18" t="n">
-        <v>0</v>
-      </c>
-      <c r="X18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA18" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>9</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT18" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV18" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AW18" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B19" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>1741255</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>EVELYN GOMEZ LOZANO</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>10223</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" t="n">
-        <v>4</v>
-      </c>
-      <c r="T19" t="n">
-        <v>4</v>
-      </c>
-      <c r="U19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" t="n">
-        <v>0</v>
-      </c>
-      <c r="X19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ19" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK19" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL19" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>9</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT19" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AW19" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B20" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>1665372</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>DORIS ANGARITA</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>10260</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AB20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="AD20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AM20" t="n">
-        <v>7</v>
-      </c>
-      <c r="AN20" t="n">
-        <v>9</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT20" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV20" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AW20" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>202612</v>
-      </c>
-      <c r="B21" t="n">
-        <v>700000003</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>GERENCIA VENTAS ARTE KARENTH</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>700000459</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SECTOR MATICES CLERY</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>985990</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>MARIA CRISTINA RUBIO</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>ORO</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>9400</v>
-      </c>
-      <c r="J21" t="n">
-        <v>23747542.18</v>
-      </c>
-      <c r="K21" t="n">
-        <v>1573859</v>
-      </c>
-      <c r="L21" t="n">
-        <v>6.627460593903027</v>
-      </c>
-      <c r="M21" t="n">
-        <v>68</v>
-      </c>
-      <c r="N21" t="n">
-        <v>5</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="n">
-        <v>-11</v>
-      </c>
-      <c r="S21" t="n">
-        <v>94</v>
-      </c>
-      <c r="T21" t="n">
-        <v>59</v>
-      </c>
-      <c r="U21" t="n">
-        <v>17</v>
-      </c>
-      <c r="V21" t="n">
-        <v>13</v>
-      </c>
-      <c r="W21" t="n">
-        <v>12</v>
-      </c>
-      <c r="X21" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>9</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>5.32%</t>
-        </is>
-      </c>
-      <c r="AB21" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>5.32%</t>
-        </is>
-      </c>
-      <c r="AD21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>314771.8</v>
-      </c>
-      <c r="AG21" t="n">
-        <v>11017.013</v>
-      </c>
-      <c r="AH21" t="n">
-        <v>6.63</v>
-      </c>
-      <c r="AI21" t="n">
-        <v>1573859</v>
-      </c>
-      <c r="AJ21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK21" t="n">
-        <v>8</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>10</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>12</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>14</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ21" t="n">
-        <v>22173683.18</v>
-      </c>
-      <c r="AR21" t="n">
-        <v>22173683.18</v>
-      </c>
-      <c r="AS21" t="n">
-        <v>24548437.398</v>
-      </c>
-      <c r="AT21" t="n">
-        <v>0.009999999999999998</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>15738.59</v>
-      </c>
-      <c r="AV21" t="n">
-        <v>-0.3</v>
-      </c>
-      <c r="AW21" t="n">
         <v>-4721.576999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
actualizacion cuadro de inicios y reicinios
</commit_message>
<xml_diff>
--- a/Resultado_Metas_Procesadas.xlsx
+++ b/Resultado_Metas_Procesadas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="92">
   <si>
     <t>Ciclo</t>
   </si>
@@ -161,6 +161,12 @@
   </si>
   <si>
     <t>Potencializador_COP</t>
+  </si>
+  <si>
+    <t>Meta Inicios + Reinicios</t>
+  </si>
+  <si>
+    <t>Meta Recuperos</t>
   </si>
   <si>
     <t>GERENCIA VENTAS ARTE KARENTH</t>
@@ -615,10 +621,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AW15"/>
+  <dimension ref="A1:AY15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:49">
+    <row r="1" spans="1:51">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -766,8 +772,14 @@
       <c r="AW1" t="s">
         <v>48</v>
       </c>
+      <c r="AX1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="2" spans="1:49">
+    <row r="2" spans="1:51">
       <c r="A2">
         <v>202612</v>
       </c>
@@ -775,22 +787,22 @@
         <v>700000003</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2">
         <v>700000459</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F2">
         <v>1694138</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I2">
         <v>9640</v>
@@ -847,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="AA2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="AB2">
         <v>11</v>
       </c>
       <c r="AC2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="AD2">
         <v>2</v>
@@ -915,8 +927,14 @@
       <c r="AW2">
         <v>-8318.891999999998</v>
       </c>
+      <c r="AX2">
+        <v>0</v>
+      </c>
+      <c r="AY2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:49">
+    <row r="3" spans="1:51">
       <c r="A3">
         <v>202612</v>
       </c>
@@ -924,19 +942,19 @@
         <v>700000003</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D3">
         <v>700000459</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F3">
         <v>1099653</v>
       </c>
       <c r="G3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I3">
         <v>9334</v>
@@ -993,13 +1011,13 @@
         <v>3</v>
       </c>
       <c r="AA3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AB3">
         <v>69</v>
       </c>
       <c r="AC3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AD3">
         <v>4</v>
@@ -1061,8 +1079,14 @@
       <c r="AW3">
         <v>-153473.616</v>
       </c>
+      <c r="AX3">
+        <v>7</v>
+      </c>
+      <c r="AY3">
+        <v>6</v>
+      </c>
     </row>
-    <row r="4" spans="1:49">
+    <row r="4" spans="1:51">
       <c r="A4">
         <v>202612</v>
       </c>
@@ -1070,22 +1094,22 @@
         <v>700000003</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D4">
         <v>700000459</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F4">
         <v>1021104</v>
       </c>
       <c r="G4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I4">
         <v>7841</v>
@@ -1142,13 +1166,13 @@
         <v>2</v>
       </c>
       <c r="AA4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AB4">
         <v>118</v>
       </c>
       <c r="AC4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AD4">
         <v>3</v>
@@ -1210,8 +1234,14 @@
       <c r="AW4">
         <v>-145517.934</v>
       </c>
+      <c r="AX4">
+        <v>7</v>
+      </c>
+      <c r="AY4">
+        <v>6</v>
+      </c>
     </row>
-    <row r="5" spans="1:49">
+    <row r="5" spans="1:51">
       <c r="A5">
         <v>202612</v>
       </c>
@@ -1219,22 +1249,22 @@
         <v>700000003</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D5">
         <v>700000459</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F5">
         <v>800685</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I5">
         <v>10168</v>
@@ -1291,13 +1321,13 @@
         <v>0</v>
       </c>
       <c r="AA5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AB5">
         <v>4</v>
       </c>
       <c r="AC5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD5">
         <v>5</v>
@@ -1359,8 +1389,14 @@
       <c r="AW5">
         <v>6070.806</v>
       </c>
+      <c r="AX5">
+        <v>0</v>
+      </c>
+      <c r="AY5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:49">
+    <row r="6" spans="1:51">
       <c r="A6">
         <v>202612</v>
       </c>
@@ -1368,19 +1404,19 @@
         <v>700000003</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D6">
         <v>700000459</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F6">
         <v>1407710</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I6">
         <v>9678</v>
@@ -1437,13 +1473,13 @@
         <v>0</v>
       </c>
       <c r="AA6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="AB6">
         <v>3</v>
       </c>
       <c r="AC6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="AD6">
         <v>0</v>
@@ -1505,8 +1541,14 @@
       <c r="AW6">
         <v>-0</v>
       </c>
+      <c r="AX6">
+        <v>0</v>
+      </c>
+      <c r="AY6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:49">
+    <row r="7" spans="1:51">
       <c r="A7">
         <v>202612</v>
       </c>
@@ -1514,22 +1556,22 @@
         <v>700000003</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D7">
         <v>700000459</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F7">
         <v>1077740</v>
       </c>
       <c r="G7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I7">
         <v>9291</v>
@@ -1586,13 +1628,13 @@
         <v>4</v>
       </c>
       <c r="AA7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="AB7">
         <v>59</v>
       </c>
       <c r="AC7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AD7">
         <v>1</v>
@@ -1654,8 +1696,14 @@
       <c r="AW7">
         <v>0</v>
       </c>
+      <c r="AX7">
+        <v>4</v>
+      </c>
+      <c r="AY7">
+        <v>5</v>
+      </c>
     </row>
-    <row r="8" spans="1:49">
+    <row r="8" spans="1:51">
       <c r="A8">
         <v>202612</v>
       </c>
@@ -1663,22 +1711,22 @@
         <v>700000003</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D8">
         <v>700000459</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F8">
         <v>813431</v>
       </c>
       <c r="G8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I8">
         <v>8425</v>
@@ -1735,13 +1783,13 @@
         <v>6</v>
       </c>
       <c r="AA8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="AB8">
         <v>109</v>
       </c>
       <c r="AC8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AD8">
         <v>1</v>
@@ -1803,8 +1851,14 @@
       <c r="AW8">
         <v>-190153.341</v>
       </c>
+      <c r="AX8">
+        <v>13</v>
+      </c>
+      <c r="AY8">
+        <v>9</v>
+      </c>
     </row>
-    <row r="9" spans="1:49">
+    <row r="9" spans="1:51">
       <c r="A9">
         <v>202612</v>
       </c>
@@ -1812,22 +1866,22 @@
         <v>700000003</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D9">
         <v>700000459</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F9">
         <v>1297183</v>
       </c>
       <c r="G9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I9">
         <v>9948</v>
@@ -1884,13 +1938,13 @@
         <v>0</v>
       </c>
       <c r="AA9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AB9">
         <v>7</v>
       </c>
       <c r="AC9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD9">
         <v>1</v>
@@ -1952,8 +2006,14 @@
       <c r="AW9">
         <v>-6075.661999999999</v>
       </c>
+      <c r="AX9">
+        <v>0</v>
+      </c>
+      <c r="AY9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:49">
+    <row r="10" spans="1:51">
       <c r="A10">
         <v>202612</v>
       </c>
@@ -1961,19 +2021,19 @@
         <v>700000003</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D10">
         <v>700000459</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F10">
         <v>1019466</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I10">
         <v>9717</v>
@@ -2030,13 +2090,13 @@
         <v>1</v>
       </c>
       <c r="AA10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AB10">
         <v>1</v>
       </c>
       <c r="AC10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AD10">
         <v>0</v>
@@ -2098,8 +2158,14 @@
       <c r="AW10">
         <v>-0</v>
       </c>
+      <c r="AX10">
+        <v>0</v>
+      </c>
+      <c r="AY10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:49">
+    <row r="11" spans="1:51">
       <c r="A11">
         <v>202612</v>
       </c>
@@ -2107,19 +2173,19 @@
         <v>700000003</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D11">
         <v>700000459</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F11">
         <v>768496</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I11">
         <v>8481</v>
@@ -2176,13 +2242,13 @@
         <v>2</v>
       </c>
       <c r="AA11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="AB11">
         <v>98</v>
       </c>
       <c r="AC11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AD11">
         <v>2</v>
@@ -2244,8 +2310,14 @@
       <c r="AW11">
         <v>-153253.50003</v>
       </c>
+      <c r="AX11">
+        <v>6</v>
+      </c>
+      <c r="AY11">
+        <v>8</v>
+      </c>
     </row>
-    <row r="12" spans="1:49">
+    <row r="12" spans="1:51">
       <c r="A12">
         <v>202612</v>
       </c>
@@ -2253,19 +2325,19 @@
         <v>700000003</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D12">
         <v>700000459</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F12">
         <v>1756380</v>
       </c>
       <c r="G12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I12">
         <v>10255</v>
@@ -2322,13 +2394,13 @@
         <v>0</v>
       </c>
       <c r="AA12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AB12">
         <v>1</v>
       </c>
       <c r="AC12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AD12">
         <v>0</v>
@@ -2390,8 +2462,14 @@
       <c r="AW12">
         <v>-516.4679999999998</v>
       </c>
+      <c r="AX12">
+        <v>0</v>
+      </c>
+      <c r="AY12">
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:49">
+    <row r="13" spans="1:51">
       <c r="A13">
         <v>202612</v>
       </c>
@@ -2399,22 +2477,22 @@
         <v>700000003</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D13">
         <v>700000459</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F13">
         <v>1741255</v>
       </c>
       <c r="G13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I13">
         <v>10223</v>
@@ -2471,13 +2549,13 @@
         <v>0</v>
       </c>
       <c r="AA13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AB13">
         <v>3</v>
       </c>
       <c r="AC13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="AD13">
         <v>2</v>
@@ -2539,8 +2617,14 @@
       <c r="AW13">
         <v>0</v>
       </c>
+      <c r="AX13">
+        <v>0</v>
+      </c>
+      <c r="AY13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:49">
+    <row r="14" spans="1:51">
       <c r="A14">
         <v>202612</v>
       </c>
@@ -2548,22 +2632,22 @@
         <v>700000003</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D14">
         <v>700000459</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F14">
         <v>1665372</v>
       </c>
       <c r="G14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H14" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I14">
         <v>10260</v>
@@ -2620,13 +2704,13 @@
         <v>0</v>
       </c>
       <c r="AA14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AB14">
         <v>1</v>
       </c>
       <c r="AC14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AD14">
         <v>1</v>
@@ -2688,8 +2772,14 @@
       <c r="AW14">
         <v>0</v>
       </c>
+      <c r="AX14">
+        <v>0</v>
+      </c>
+      <c r="AY14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:49">
+    <row r="15" spans="1:51">
       <c r="A15">
         <v>202612</v>
       </c>
@@ -2697,22 +2787,22 @@
         <v>700000003</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D15">
         <v>700000459</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F15">
         <v>985990</v>
       </c>
       <c r="G15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I15">
         <v>9400</v>
@@ -2769,13 +2859,13 @@
         <v>1</v>
       </c>
       <c r="AA15" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AB15">
         <v>36</v>
       </c>
       <c r="AC15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AD15">
         <v>2</v>
@@ -2836,6 +2926,12 @@
       </c>
       <c r="AW15">
         <v>-38280.46799999999</v>
+      </c>
+      <c r="AX15">
+        <v>5</v>
+      </c>
+      <c r="AY15">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>